<commit_message>
Add Graham Barber to Thursday VOFF Cloud wks 10-13 (closes gap)
</commit_message>
<xml_diff>
--- a/output/teacher_timetables_S2_2026.xlsx
+++ b/output/teacher_timetables_S2_2026.xlsx
@@ -142,7 +142,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">8</t>
+          <t xml:space="preserve">9</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -152,17 +152,17 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t xml:space="preserve">14</t>
+          <t xml:space="preserve">16</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t xml:space="preserve">28.0</t>
+          <t xml:space="preserve">33.5</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t xml:space="preserve">273.0</t>
+          <t xml:space="preserve">295.0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -2128,7 +2128,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">50</t>
+          <t xml:space="preserve">51</t>
         </is>
       </c>
     </row>
@@ -2164,7 +2164,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">5</t>
+          <t xml:space="preserve">6</t>
         </is>
       </c>
     </row>
@@ -2561,24 +2561,24 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">COMBINED-MERGE</t>
+          <t xml:space="preserve">ADJ-APPLIED</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jennie Agustin Wednesday 2:30-3:30 tutorial: merged F2F+VOFF into one (Cert III General (F2F+VOFF combined)), counted once.</t>
+          <t xml:space="preserve">GRAHAM-1 [add_teacher] Graham Barber on [Cert III General (VOFF)] Thursday 9:00-2:30 (ICTCLD301): Graham Barber covers the Thursday VOFF (Cloud) session wks 10-13, before Anu takes over from wk14. Closes the wks 10-13 gap.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO-TEACHER</t>
+          <t xml:space="preserve">COMBINED-MERGE</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">[Cert IV VOCF] Wednesday 3:30-5:00 Tutorial Support: Optional Tutorial support combined with Diploma Group</t>
+          <t xml:space="preserve">Jennie Agustin Wednesday 2:30-3:30 tutorial: merged F2F+VOFF into one (Cert III General (F2F+VOFF combined)), counted once.</t>
         </is>
       </c>
     </row>
@@ -2590,7 +2590,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">[Cert IV VOCF] Thursday 12:30-2:30 Self-directed learning: Self-directed learning</t>
+          <t xml:space="preserve">[Cert IV VOCF] Wednesday 3:30-5:00 Tutorial Support: Optional Tutorial support combined with Diploma Group</t>
         </is>
       </c>
     </row>
@@ -2602,7 +2602,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">[Diploma Library Services - Fulltime VOFF] Wednesday 3:30pm-5:00pm Tutorial Support: Tutorial time</t>
+          <t xml:space="preserve">[Cert IV VOCF] Thursday 12:30-2:30 Self-directed learning: Self-directed learning</t>
         </is>
       </c>
     </row>
@@ -2614,7 +2614,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">[Cert III General (F2F)] Tuesday 9:00-2:30 Teaching: ICTCLD301 Evaluate Characteristics of Cloud Computing Solutions and services. | BSBXCS303 Securely manage personally identifiable information and workplace information. | ICTICT313 Identify IP, ethics, and privacy policies in ICT environments.</t>
+          <t xml:space="preserve">[Diploma Library Services - Fulltime VOFF] Wednesday 3:30pm-5:00pm Tutorial Support: Tutorial time</t>
         </is>
       </c>
     </row>
@@ -2626,7 +2626,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">[Cert III General (F2F)] Tuesday 2:30-3:30 Tutorial Support: Tutorial Support</t>
+          <t xml:space="preserve">[Cert III General (F2F)] Tuesday 9:00-2:30 Teaching: ICTCLD301 Evaluate Characteristics of Cloud Computing Solutions and services. | BSBXCS303 Securely manage personally identifiable information and workplace information. | ICTICT313 Identify IP, ethics, and privacy policies in ICT environments.</t>
         </is>
       </c>
     </row>
@@ -2638,7 +2638,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">[Cert III General (F2F)] Thursday 9:00-2:30 Teaching: ICTPRG302 Apply introductory programming techniques.</t>
+          <t xml:space="preserve">[Cert III General (F2F)] Tuesday 2:30-3:30 Tutorial Support: Tutorial Support</t>
         </is>
       </c>
     </row>
@@ -2649,6 +2649,18 @@
         </is>
       </c>
       <c r="B14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[Cert III General (F2F)] Thursday 9:00-2:30 Teaching: ICTPRG302 Apply introductory programming techniques.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO-TEACHER</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
         <is>
           <t xml:space="preserve">[Cert III General (VOFF)] Tuesday 9:00-2:30 Teaching: BSBCRT301 Develop and extend critical and creative thinking skills. | BSBXTW301 Work in a team. | ICTSAS305 Provide ICT advice to clients.</t>
         </is>
@@ -2917,7 +2929,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Graham Barber</t>
         </is>
       </c>
     </row>
@@ -3559,6 +3571,58 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Thursday</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9:00-2:30</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10-13</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5.5</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">22.0</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cert III General (VOFF)</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VOFF</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Teaching</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ICTCLD301 Evaluate Characteristics of Cloud Computing solutions and services | ICTICT310 Identify and use industry specific technologies.</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Anu Joshi</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Fix: list a co-teacher only when their weeks overlap (hand-over is not co-teaching)
</commit_message>
<xml_diff>
--- a/output/teacher_timetables_S2_2026.xlsx
+++ b/output/teacher_timetables_S2_2026.xlsx
@@ -1650,7 +1650,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jennie Agustin</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -2929,7 +2929,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Graham Barber</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -3619,7 +3619,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Anu Joshi</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -3834,7 +3834,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Shanna Roper</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>

</xml_diff>